<commit_message>
script write to migrate data in mba sem
</commit_message>
<xml_diff>
--- a/courses_data/mba/MBA_Result.xlsx
+++ b/courses_data/mba/MBA_Result.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
   <si>
     <t xml:space="preserve">                                                         Purnea University, Purnia, Bihar</t>
   </si>
@@ -151,45 +151,14 @@
   </si>
   <si>
     <t xml:space="preserve">Pass Marks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANWAR ALI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1911B320024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ABHISHEK KUMAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2311M230001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SHALINI SHEKHAR K S RANJAN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2311M230002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMARDEEP KUMAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2311M230003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SANYA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2311M230004</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -360,7 +329,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -421,10 +390,6 @@
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -434,10 +399,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -516,9 +477,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>27</xdr:col>
-      <xdr:colOff>94320</xdr:colOff>
+      <xdr:colOff>93600</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>1171800</xdr:rowOff>
+      <xdr:rowOff>1171080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -532,7 +493,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9858600" y="207360"/>
-          <a:ext cx="960120" cy="964440"/>
+          <a:ext cx="959400" cy="963720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1503,763 +1464,668 @@
       <c r="AZ15" s="14"/>
     </row>
     <row r="16" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="n">
+      <c r="A16" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="C16" s="15" t="n">
+      <c r="C16" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D16" s="15" t="n">
+      <c r="D16" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E16" s="15" t="n">
+      <c r="E16" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="F16" s="15" t="n">
+      <c r="F16" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="G16" s="15" t="n">
+      <c r="G16" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="H16" s="15" t="n">
+      <c r="H16" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="I16" s="15" t="n">
+      <c r="I16" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="J16" s="15" t="n">
+      <c r="J16" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="K16" s="15" t="n">
+      <c r="K16" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="L16" s="15" t="n">
+      <c r="L16" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="M16" s="15" t="n">
+      <c r="M16" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="N16" s="15" t="n">
+      <c r="N16" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="O16" s="15" t="n">
+      <c r="O16" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="P16" s="15" t="n">
+      <c r="P16" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="Q16" s="15" t="n">
+      <c r="Q16" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="R16" s="15" t="n">
+      <c r="R16" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="S16" s="15" t="n">
+      <c r="S16" s="10" t="n">
         <v>19</v>
       </c>
-      <c r="T16" s="15" t="n">
+      <c r="T16" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="U16" s="15" t="n">
+      <c r="U16" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="V16" s="15" t="n">
+      <c r="V16" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="W16" s="15" t="n">
+      <c r="W16" s="10" t="n">
         <v>23</v>
       </c>
-      <c r="X16" s="15" t="n">
+      <c r="X16" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="Y16" s="15" t="n">
+      <c r="Y16" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="Z16" s="15" t="n">
+      <c r="Z16" s="10" t="n">
         <v>26</v>
       </c>
-      <c r="AA16" s="15" t="n">
+      <c r="AA16" s="10" t="n">
         <v>27</v>
       </c>
-      <c r="AB16" s="15" t="n">
+      <c r="AB16" s="10" t="n">
         <v>28</v>
       </c>
-      <c r="AC16" s="15" t="n">
+      <c r="AC16" s="10" t="n">
         <v>29</v>
       </c>
-      <c r="AD16" s="15" t="n">
+      <c r="AD16" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="AE16" s="15" t="n">
+      <c r="AE16" s="10" t="n">
         <v>31</v>
       </c>
-      <c r="AF16" s="15" t="n">
+      <c r="AF16" s="10" t="n">
         <v>32</v>
       </c>
-      <c r="AG16" s="15" t="n">
+      <c r="AG16" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="AH16" s="15" t="n">
+      <c r="AH16" s="10" t="n">
         <v>34</v>
       </c>
-      <c r="AI16" s="15" t="n">
+      <c r="AI16" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="AJ16" s="15" t="n">
+      <c r="AJ16" s="10" t="n">
         <v>36</v>
       </c>
-      <c r="AK16" s="15" t="n">
+      <c r="AK16" s="10" t="n">
         <v>37</v>
       </c>
-      <c r="AL16" s="15" t="n">
+      <c r="AL16" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="AM16" s="15" t="n">
+      <c r="AM16" s="10" t="n">
         <v>39</v>
       </c>
-      <c r="AN16" s="15" t="n">
+      <c r="AN16" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="AO16" s="15" t="n">
+      <c r="AO16" s="10" t="n">
         <v>41</v>
       </c>
-      <c r="AP16" s="15" t="n">
+      <c r="AP16" s="10" t="n">
         <v>42</v>
       </c>
-      <c r="AQ16" s="15" t="n">
+      <c r="AQ16" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="AR16" s="15" t="n">
+      <c r="AR16" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="AS16" s="15" t="n">
+      <c r="AS16" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="AT16" s="15" t="n">
+      <c r="AT16" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="AU16" s="15" t="n">
+      <c r="AU16" s="10" t="n">
         <v>47</v>
       </c>
-      <c r="AV16" s="15" t="n">
+      <c r="AV16" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="AW16" s="15" t="n">
+      <c r="AW16" s="10" t="n">
         <v>49</v>
       </c>
-      <c r="AX16" s="15" t="n">
+      <c r="AX16" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="AY16" s="15" t="n">
+      <c r="AY16" s="10" t="n">
         <v>51</v>
       </c>
-      <c r="AZ16" s="15" t="n">
+      <c r="AZ16" s="10" t="n">
         <v>52</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="57.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="16" t="n">
-        <v>8115</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="17"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
-      <c r="P17" s="17"/>
-      <c r="Q17" s="17"/>
-      <c r="R17" s="17"/>
-      <c r="S17" s="17"/>
-      <c r="T17" s="17"/>
-      <c r="U17" s="17"/>
-      <c r="V17" s="17"/>
-      <c r="W17" s="17"/>
-      <c r="X17" s="17"/>
-      <c r="Y17" s="17"/>
-      <c r="Z17" s="17"/>
-      <c r="AA17" s="17"/>
-      <c r="AB17" s="17"/>
-      <c r="AC17" s="17"/>
-      <c r="AD17" s="17"/>
-      <c r="AE17" s="17"/>
-      <c r="AF17" s="17"/>
-      <c r="AG17" s="17"/>
-      <c r="AH17" s="17"/>
-      <c r="AI17" s="17"/>
-      <c r="AJ17" s="17"/>
-      <c r="AK17" s="17"/>
-      <c r="AL17" s="17"/>
-      <c r="AM17" s="17"/>
-      <c r="AN17" s="17"/>
-      <c r="AO17" s="17"/>
-      <c r="AP17" s="17"/>
-      <c r="AQ17" s="17"/>
-      <c r="AR17" s="17"/>
-      <c r="AS17" s="17"/>
-      <c r="AT17" s="17"/>
-      <c r="AU17" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="AV17" s="18" t="n">
-        <v>24</v>
-      </c>
-      <c r="AW17" s="19" t="n">
-        <f aca="false">192/24</f>
-        <v>8</v>
-      </c>
-      <c r="AX17" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="AY17" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="AZ17" s="17" t="s">
-        <v>32</v>
-      </c>
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="16"/>
+      <c r="N17" s="16"/>
+      <c r="O17" s="16"/>
+      <c r="P17" s="16"/>
+      <c r="Q17" s="16"/>
+      <c r="R17" s="16"/>
+      <c r="S17" s="16"/>
+      <c r="T17" s="16"/>
+      <c r="U17" s="16"/>
+      <c r="V17" s="16"/>
+      <c r="W17" s="16"/>
+      <c r="X17" s="16"/>
+      <c r="Y17" s="16"/>
+      <c r="Z17" s="16"/>
+      <c r="AA17" s="16"/>
+      <c r="AB17" s="16"/>
+      <c r="AC17" s="16"/>
+      <c r="AD17" s="16"/>
+      <c r="AE17" s="16"/>
+      <c r="AF17" s="16"/>
+      <c r="AG17" s="16"/>
+      <c r="AH17" s="16"/>
+      <c r="AI17" s="16"/>
+      <c r="AJ17" s="16"/>
+      <c r="AK17" s="16"/>
+      <c r="AL17" s="16"/>
+      <c r="AM17" s="16"/>
+      <c r="AN17" s="16"/>
+      <c r="AO17" s="16"/>
+      <c r="AP17" s="16"/>
+      <c r="AQ17" s="16"/>
+      <c r="AR17" s="16"/>
+      <c r="AS17" s="16"/>
+      <c r="AT17" s="16"/>
+      <c r="AU17" s="16"/>
+      <c r="AV17" s="17"/>
+      <c r="AW17" s="13"/>
+      <c r="AX17" s="16"/>
+      <c r="AY17" s="16"/>
+      <c r="AZ17" s="16"/>
     </row>
     <row r="18" customFormat="false" ht="57.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16" t="n">
-        <v>8116</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="17"/>
-      <c r="O18" s="17"/>
-      <c r="P18" s="17"/>
-      <c r="Q18" s="17"/>
-      <c r="R18" s="17"/>
-      <c r="S18" s="17"/>
-      <c r="T18" s="17"/>
-      <c r="U18" s="17"/>
-      <c r="V18" s="17"/>
-      <c r="W18" s="17"/>
-      <c r="X18" s="17"/>
-      <c r="Y18" s="17"/>
-      <c r="Z18" s="17"/>
-      <c r="AA18" s="17"/>
-      <c r="AB18" s="17"/>
-      <c r="AC18" s="17"/>
-      <c r="AD18" s="17"/>
-      <c r="AE18" s="17"/>
-      <c r="AF18" s="17"/>
-      <c r="AG18" s="17"/>
-      <c r="AH18" s="17"/>
-      <c r="AI18" s="17"/>
-      <c r="AJ18" s="17"/>
-      <c r="AK18" s="17"/>
-      <c r="AL18" s="17"/>
-      <c r="AM18" s="17"/>
-      <c r="AN18" s="17"/>
-      <c r="AO18" s="17"/>
-      <c r="AP18" s="17"/>
-      <c r="AQ18" s="17"/>
-      <c r="AR18" s="17"/>
-      <c r="AS18" s="17"/>
-      <c r="AT18" s="17"/>
-      <c r="AU18" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="AV18" s="18" t="n">
-        <v>24</v>
-      </c>
-      <c r="AW18" s="19" t="n">
-        <f aca="false">192/24</f>
-        <v>8</v>
-      </c>
-      <c r="AX18" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="AY18" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="AZ18" s="17" t="s">
-        <v>32</v>
-      </c>
+      <c r="A18" s="15"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16"/>
+      <c r="P18" s="16"/>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="16"/>
+      <c r="S18" s="16"/>
+      <c r="T18" s="16"/>
+      <c r="U18" s="16"/>
+      <c r="V18" s="16"/>
+      <c r="W18" s="16"/>
+      <c r="X18" s="16"/>
+      <c r="Y18" s="16"/>
+      <c r="Z18" s="16"/>
+      <c r="AA18" s="16"/>
+      <c r="AB18" s="16"/>
+      <c r="AC18" s="16"/>
+      <c r="AD18" s="16"/>
+      <c r="AE18" s="16"/>
+      <c r="AF18" s="16"/>
+      <c r="AG18" s="16"/>
+      <c r="AH18" s="16"/>
+      <c r="AI18" s="16"/>
+      <c r="AJ18" s="16"/>
+      <c r="AK18" s="16"/>
+      <c r="AL18" s="16"/>
+      <c r="AM18" s="16"/>
+      <c r="AN18" s="16"/>
+      <c r="AO18" s="16"/>
+      <c r="AP18" s="16"/>
+      <c r="AQ18" s="16"/>
+      <c r="AR18" s="16"/>
+      <c r="AS18" s="16"/>
+      <c r="AT18" s="16"/>
+      <c r="AU18" s="16"/>
+      <c r="AV18" s="17"/>
+      <c r="AW18" s="13"/>
+      <c r="AX18" s="16"/>
+      <c r="AY18" s="16"/>
+      <c r="AZ18" s="16"/>
     </row>
     <row r="19" customFormat="false" ht="57.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="16" t="n">
-        <v>8117</v>
-      </c>
-      <c r="B19" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="C19" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="17"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="17"/>
-      <c r="M19" s="17"/>
-      <c r="N19" s="17"/>
-      <c r="O19" s="17"/>
-      <c r="P19" s="17"/>
-      <c r="Q19" s="17"/>
-      <c r="R19" s="17"/>
-      <c r="S19" s="17"/>
-      <c r="T19" s="17"/>
-      <c r="U19" s="17"/>
-      <c r="V19" s="17"/>
-      <c r="W19" s="17"/>
-      <c r="X19" s="17"/>
-      <c r="Y19" s="17"/>
-      <c r="Z19" s="17"/>
-      <c r="AA19" s="17"/>
-      <c r="AB19" s="17"/>
-      <c r="AC19" s="17"/>
-      <c r="AD19" s="17"/>
-      <c r="AE19" s="17"/>
-      <c r="AF19" s="17"/>
-      <c r="AG19" s="17"/>
-      <c r="AH19" s="17"/>
-      <c r="AI19" s="17"/>
-      <c r="AJ19" s="17"/>
-      <c r="AK19" s="17"/>
-      <c r="AL19" s="17"/>
-      <c r="AM19" s="17"/>
-      <c r="AN19" s="17"/>
-      <c r="AO19" s="17"/>
-      <c r="AP19" s="17"/>
-      <c r="AQ19" s="17"/>
-      <c r="AR19" s="17"/>
-      <c r="AS19" s="17"/>
-      <c r="AT19" s="17"/>
-      <c r="AU19" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="AV19" s="18" t="n">
-        <v>24</v>
-      </c>
-      <c r="AW19" s="19" t="n">
-        <f aca="false">192/24</f>
-        <v>8</v>
-      </c>
-      <c r="AX19" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="AY19" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="AZ19" s="17" t="s">
-        <v>32</v>
-      </c>
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
+      <c r="M19" s="16"/>
+      <c r="N19" s="16"/>
+      <c r="O19" s="16"/>
+      <c r="P19" s="16"/>
+      <c r="Q19" s="16"/>
+      <c r="R19" s="16"/>
+      <c r="S19" s="16"/>
+      <c r="T19" s="16"/>
+      <c r="U19" s="16"/>
+      <c r="V19" s="16"/>
+      <c r="W19" s="16"/>
+      <c r="X19" s="16"/>
+      <c r="Y19" s="16"/>
+      <c r="Z19" s="16"/>
+      <c r="AA19" s="16"/>
+      <c r="AB19" s="16"/>
+      <c r="AC19" s="16"/>
+      <c r="AD19" s="16"/>
+      <c r="AE19" s="16"/>
+      <c r="AF19" s="16"/>
+      <c r="AG19" s="16"/>
+      <c r="AH19" s="16"/>
+      <c r="AI19" s="16"/>
+      <c r="AJ19" s="16"/>
+      <c r="AK19" s="16"/>
+      <c r="AL19" s="16"/>
+      <c r="AM19" s="16"/>
+      <c r="AN19" s="16"/>
+      <c r="AO19" s="16"/>
+      <c r="AP19" s="16"/>
+      <c r="AQ19" s="16"/>
+      <c r="AR19" s="16"/>
+      <c r="AS19" s="16"/>
+      <c r="AT19" s="16"/>
+      <c r="AU19" s="16"/>
+      <c r="AV19" s="17"/>
+      <c r="AW19" s="13"/>
+      <c r="AX19" s="16"/>
+      <c r="AY19" s="16"/>
+      <c r="AZ19" s="16"/>
     </row>
     <row r="20" customFormat="false" ht="57.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="16" t="n">
-        <v>8118</v>
-      </c>
-      <c r="B20" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="17"/>
-      <c r="M20" s="17"/>
-      <c r="N20" s="17"/>
-      <c r="O20" s="17"/>
-      <c r="P20" s="17"/>
-      <c r="Q20" s="17"/>
-      <c r="R20" s="17"/>
-      <c r="S20" s="17"/>
-      <c r="T20" s="17"/>
-      <c r="U20" s="17"/>
-      <c r="V20" s="17"/>
-      <c r="W20" s="17"/>
-      <c r="X20" s="17"/>
-      <c r="Y20" s="17"/>
-      <c r="Z20" s="17"/>
-      <c r="AA20" s="17"/>
-      <c r="AB20" s="17"/>
-      <c r="AC20" s="17"/>
-      <c r="AD20" s="17"/>
-      <c r="AE20" s="17"/>
-      <c r="AF20" s="17"/>
-      <c r="AG20" s="17"/>
-      <c r="AH20" s="17"/>
-      <c r="AI20" s="17"/>
-      <c r="AJ20" s="17"/>
-      <c r="AK20" s="17"/>
-      <c r="AL20" s="17"/>
-      <c r="AM20" s="17"/>
-      <c r="AN20" s="17"/>
-      <c r="AO20" s="17"/>
-      <c r="AP20" s="17"/>
-      <c r="AQ20" s="17"/>
-      <c r="AR20" s="17"/>
-      <c r="AS20" s="17"/>
-      <c r="AT20" s="17"/>
-      <c r="AU20" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="AV20" s="18" t="n">
-        <v>24</v>
-      </c>
-      <c r="AW20" s="19" t="n">
-        <f aca="false">192/24</f>
-        <v>8</v>
-      </c>
-      <c r="AX20" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="AY20" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="AZ20" s="17" t="s">
-        <v>32</v>
-      </c>
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
+      <c r="M20" s="16"/>
+      <c r="N20" s="16"/>
+      <c r="O20" s="16"/>
+      <c r="P20" s="16"/>
+      <c r="Q20" s="16"/>
+      <c r="R20" s="16"/>
+      <c r="S20" s="16"/>
+      <c r="T20" s="16"/>
+      <c r="U20" s="16"/>
+      <c r="V20" s="16"/>
+      <c r="W20" s="16"/>
+      <c r="X20" s="16"/>
+      <c r="Y20" s="16"/>
+      <c r="Z20" s="16"/>
+      <c r="AA20" s="16"/>
+      <c r="AB20" s="16"/>
+      <c r="AC20" s="16"/>
+      <c r="AD20" s="16"/>
+      <c r="AE20" s="16"/>
+      <c r="AF20" s="16"/>
+      <c r="AG20" s="16"/>
+      <c r="AH20" s="16"/>
+      <c r="AI20" s="16"/>
+      <c r="AJ20" s="16"/>
+      <c r="AK20" s="16"/>
+      <c r="AL20" s="16"/>
+      <c r="AM20" s="16"/>
+      <c r="AN20" s="16"/>
+      <c r="AO20" s="16"/>
+      <c r="AP20" s="16"/>
+      <c r="AQ20" s="16"/>
+      <c r="AR20" s="16"/>
+      <c r="AS20" s="16"/>
+      <c r="AT20" s="16"/>
+      <c r="AU20" s="16"/>
+      <c r="AV20" s="17"/>
+      <c r="AW20" s="13"/>
+      <c r="AX20" s="16"/>
+      <c r="AY20" s="16"/>
+      <c r="AZ20" s="16"/>
     </row>
     <row r="21" customFormat="false" ht="57.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="16" t="n">
-        <v>8119</v>
-      </c>
-      <c r="B21" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="17"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="17"/>
-      <c r="K21" s="17"/>
-      <c r="L21" s="17"/>
-      <c r="M21" s="17"/>
-      <c r="N21" s="17"/>
-      <c r="O21" s="17"/>
-      <c r="P21" s="17"/>
-      <c r="Q21" s="17"/>
-      <c r="R21" s="17"/>
-      <c r="S21" s="17"/>
-      <c r="T21" s="17"/>
-      <c r="U21" s="17"/>
-      <c r="V21" s="17"/>
-      <c r="W21" s="17"/>
-      <c r="X21" s="17"/>
-      <c r="Y21" s="17"/>
-      <c r="Z21" s="17"/>
-      <c r="AA21" s="17"/>
-      <c r="AB21" s="17"/>
-      <c r="AC21" s="17"/>
-      <c r="AD21" s="17"/>
-      <c r="AE21" s="17"/>
-      <c r="AF21" s="17"/>
-      <c r="AG21" s="17"/>
-      <c r="AH21" s="17"/>
-      <c r="AI21" s="17"/>
-      <c r="AJ21" s="17"/>
-      <c r="AK21" s="17"/>
-      <c r="AL21" s="17"/>
-      <c r="AM21" s="17"/>
-      <c r="AN21" s="17"/>
-      <c r="AO21" s="17"/>
-      <c r="AP21" s="17"/>
-      <c r="AQ21" s="17"/>
-      <c r="AR21" s="17"/>
-      <c r="AS21" s="17"/>
-      <c r="AT21" s="17"/>
-      <c r="AU21" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="AV21" s="18" t="n">
-        <v>24</v>
-      </c>
-      <c r="AW21" s="19" t="n">
-        <f aca="false">192/24</f>
-        <v>8</v>
-      </c>
-      <c r="AX21" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="AY21" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="AZ21" s="17" t="s">
-        <v>32</v>
-      </c>
+      <c r="A21" s="15"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="16"/>
+      <c r="N21" s="16"/>
+      <c r="O21" s="16"/>
+      <c r="P21" s="16"/>
+      <c r="Q21" s="16"/>
+      <c r="R21" s="16"/>
+      <c r="S21" s="16"/>
+      <c r="T21" s="16"/>
+      <c r="U21" s="16"/>
+      <c r="V21" s="16"/>
+      <c r="W21" s="16"/>
+      <c r="X21" s="16"/>
+      <c r="Y21" s="16"/>
+      <c r="Z21" s="16"/>
+      <c r="AA21" s="16"/>
+      <c r="AB21" s="16"/>
+      <c r="AC21" s="16"/>
+      <c r="AD21" s="16"/>
+      <c r="AE21" s="16"/>
+      <c r="AF21" s="16"/>
+      <c r="AG21" s="16"/>
+      <c r="AH21" s="16"/>
+      <c r="AI21" s="16"/>
+      <c r="AJ21" s="16"/>
+      <c r="AK21" s="16"/>
+      <c r="AL21" s="16"/>
+      <c r="AM21" s="16"/>
+      <c r="AN21" s="16"/>
+      <c r="AO21" s="16"/>
+      <c r="AP21" s="16"/>
+      <c r="AQ21" s="16"/>
+      <c r="AR21" s="16"/>
+      <c r="AS21" s="16"/>
+      <c r="AT21" s="16"/>
+      <c r="AU21" s="16"/>
+      <c r="AV21" s="17"/>
+      <c r="AW21" s="13"/>
+      <c r="AX21" s="16"/>
+      <c r="AY21" s="16"/>
+      <c r="AZ21" s="16"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="AU22" s="20"/>
-      <c r="AV22" s="20"/>
-      <c r="AW22" s="21"/>
-      <c r="AX22" s="22"/>
-      <c r="AY22" s="22"/>
-      <c r="AZ22" s="22"/>
+      <c r="AU22" s="18"/>
+      <c r="AV22" s="18"/>
+      <c r="AW22" s="19"/>
+      <c r="AX22" s="20"/>
+      <c r="AY22" s="20"/>
+      <c r="AZ22" s="20"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="AU23" s="20"/>
-      <c r="AV23" s="20"/>
-      <c r="AW23" s="21"/>
-      <c r="AX23" s="22"/>
-      <c r="AY23" s="22"/>
-      <c r="AZ23" s="22"/>
+      <c r="AU23" s="18"/>
+      <c r="AV23" s="18"/>
+      <c r="AW23" s="19"/>
+      <c r="AX23" s="20"/>
+      <c r="AY23" s="20"/>
+      <c r="AZ23" s="20"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="AU24" s="20"/>
-      <c r="AV24" s="20"/>
-      <c r="AW24" s="21"/>
-      <c r="AX24" s="22"/>
-      <c r="AY24" s="22"/>
-      <c r="AZ24" s="22"/>
-    </row>
-    <row r="25" s="25" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="23"/>
-      <c r="B25" s="23"/>
-      <c r="C25" s="24"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="24"/>
-      <c r="J25" s="24"/>
-      <c r="K25" s="24"/>
-      <c r="L25" s="26"/>
-      <c r="M25" s="24"/>
-      <c r="N25" s="24"/>
-      <c r="O25" s="24"/>
-      <c r="P25" s="24"/>
-      <c r="Q25" s="26"/>
-      <c r="R25" s="24"/>
-      <c r="S25" s="24"/>
-      <c r="T25" s="26"/>
-      <c r="U25" s="24"/>
-      <c r="V25" s="24"/>
-      <c r="W25" s="24"/>
-      <c r="X25" s="24"/>
-      <c r="Y25" s="24"/>
-      <c r="Z25" s="24"/>
-      <c r="AA25" s="24"/>
-      <c r="AB25" s="26"/>
-      <c r="AC25" s="24"/>
-      <c r="AD25" s="24"/>
-      <c r="AE25" s="24"/>
-      <c r="AF25" s="24"/>
-      <c r="AG25" s="24"/>
-      <c r="AH25" s="24"/>
-      <c r="AI25" s="24"/>
-      <c r="AJ25" s="24"/>
-      <c r="AK25" s="24"/>
-      <c r="AL25" s="24"/>
-      <c r="AM25" s="24"/>
-      <c r="AN25" s="24"/>
-      <c r="AO25" s="26"/>
-      <c r="AP25" s="24"/>
-      <c r="AQ25" s="24"/>
-      <c r="AR25" s="24"/>
-      <c r="AS25" s="24"/>
-      <c r="AT25" s="24"/>
-      <c r="AU25" s="27"/>
-      <c r="AV25" s="27"/>
-      <c r="AW25" s="27"/>
-      <c r="AX25" s="24"/>
-      <c r="AY25" s="24"/>
-      <c r="AZ25" s="24"/>
-    </row>
-    <row r="26" s="25" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="23"/>
-      <c r="B26" s="24"/>
-      <c r="C26" s="24"/>
-      <c r="H26" s="24"/>
-      <c r="I26" s="24"/>
-      <c r="J26" s="24"/>
-      <c r="K26" s="24"/>
-      <c r="L26" s="26"/>
-      <c r="M26" s="24"/>
-      <c r="N26" s="24"/>
-      <c r="O26" s="24"/>
-      <c r="P26" s="24"/>
-      <c r="Q26" s="26"/>
-      <c r="R26" s="24"/>
-      <c r="S26" s="24"/>
-      <c r="T26" s="26"/>
-      <c r="U26" s="24"/>
-      <c r="V26" s="24"/>
-      <c r="W26" s="24"/>
-      <c r="X26" s="24"/>
-      <c r="Y26" s="24"/>
-      <c r="Z26" s="24"/>
-      <c r="AA26" s="24"/>
-      <c r="AB26" s="26"/>
-      <c r="AC26" s="24"/>
-      <c r="AE26" s="24"/>
-      <c r="AF26" s="24"/>
-      <c r="AG26" s="24"/>
-      <c r="AH26" s="24"/>
-      <c r="AI26" s="24"/>
-      <c r="AJ26" s="24"/>
-      <c r="AK26" s="24"/>
-      <c r="AL26" s="24"/>
-      <c r="AM26" s="24"/>
-      <c r="AN26" s="24"/>
-      <c r="AO26" s="26"/>
-      <c r="AP26" s="24"/>
-      <c r="AQ26" s="24"/>
-      <c r="AR26" s="24"/>
-      <c r="AU26" s="24"/>
-      <c r="AV26" s="24"/>
-      <c r="AW26" s="24"/>
-      <c r="AX26" s="24"/>
-      <c r="AY26" s="24"/>
-      <c r="AZ26" s="24"/>
-      <c r="BA26" s="28"/>
-      <c r="BB26" s="28"/>
-      <c r="BC26" s="24"/>
-      <c r="BD26" s="24"/>
-      <c r="BE26" s="27"/>
-    </row>
-    <row r="27" s="25" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="24"/>
-      <c r="B27" s="24"/>
-      <c r="C27" s="24"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="24"/>
-      <c r="J27" s="24"/>
-      <c r="K27" s="24"/>
-      <c r="L27" s="26"/>
-      <c r="M27" s="24"/>
-      <c r="N27" s="24"/>
-      <c r="O27" s="24"/>
-      <c r="P27" s="24"/>
-      <c r="Q27" s="26"/>
-      <c r="R27" s="24"/>
-      <c r="S27" s="24"/>
-      <c r="T27" s="26"/>
-      <c r="U27" s="24"/>
-      <c r="V27" s="24"/>
-      <c r="W27" s="24"/>
-      <c r="X27" s="24"/>
-      <c r="Y27" s="24"/>
-      <c r="Z27" s="24"/>
-      <c r="AA27" s="24"/>
-      <c r="AB27" s="26"/>
-      <c r="AC27" s="24"/>
-      <c r="AE27" s="24"/>
-      <c r="AF27" s="24"/>
-      <c r="AG27" s="24"/>
-      <c r="AH27" s="24"/>
-      <c r="AI27" s="24"/>
-      <c r="AJ27" s="24"/>
-      <c r="AK27" s="24"/>
-      <c r="AL27" s="24"/>
-      <c r="AM27" s="24"/>
-      <c r="AN27" s="24"/>
-      <c r="AO27" s="26"/>
-      <c r="AP27" s="24"/>
-      <c r="AQ27" s="24"/>
-      <c r="AR27" s="24"/>
-      <c r="AU27" s="24"/>
-      <c r="AV27" s="24"/>
-      <c r="AW27" s="24"/>
-      <c r="AX27" s="24"/>
-      <c r="AY27" s="24"/>
-      <c r="AZ27" s="24"/>
-      <c r="BA27" s="28"/>
-      <c r="BB27" s="28"/>
-      <c r="BC27" s="24"/>
-      <c r="BD27" s="24"/>
-      <c r="BE27" s="27"/>
-    </row>
-    <row r="28" s="30" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="29"/>
-      <c r="B28" s="29"/>
-      <c r="C28" s="29"/>
-      <c r="H28" s="29"/>
-      <c r="I28" s="29"/>
-      <c r="J28" s="29"/>
-      <c r="K28" s="29"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="29"/>
-      <c r="N28" s="29"/>
-      <c r="O28" s="29"/>
-      <c r="P28" s="29"/>
-      <c r="Q28" s="31"/>
-      <c r="R28" s="29"/>
-      <c r="S28" s="29"/>
-      <c r="T28" s="31"/>
-      <c r="U28" s="29"/>
-      <c r="V28" s="29"/>
-      <c r="W28" s="29"/>
-      <c r="X28" s="29"/>
-      <c r="Y28" s="29"/>
-      <c r="Z28" s="29"/>
-      <c r="AA28" s="29"/>
-      <c r="AB28" s="31"/>
-      <c r="AC28" s="29"/>
-      <c r="AD28" s="29"/>
-      <c r="AE28" s="29"/>
-      <c r="AF28" s="29"/>
-      <c r="AG28" s="29"/>
-      <c r="AH28" s="29"/>
-      <c r="AI28" s="29"/>
-      <c r="AJ28" s="29"/>
-      <c r="AK28" s="29"/>
-      <c r="AL28" s="29"/>
-      <c r="AM28" s="29"/>
-      <c r="AN28" s="29"/>
-      <c r="AO28" s="31"/>
-      <c r="AP28" s="29"/>
-      <c r="AQ28" s="29"/>
-      <c r="AR28" s="29"/>
-      <c r="AS28" s="29"/>
-      <c r="AT28" s="29"/>
-      <c r="AU28" s="21"/>
-      <c r="AV28" s="21"/>
-      <c r="AW28" s="21"/>
-      <c r="AX28" s="32"/>
-      <c r="AY28" s="32"/>
-      <c r="AZ28" s="32"/>
+      <c r="AU24" s="18"/>
+      <c r="AV24" s="18"/>
+      <c r="AW24" s="19"/>
+      <c r="AX24" s="20"/>
+      <c r="AY24" s="20"/>
+      <c r="AZ24" s="20"/>
+    </row>
+    <row r="25" s="23" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="21"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="22"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="22"/>
+      <c r="J25" s="22"/>
+      <c r="K25" s="22"/>
+      <c r="L25" s="24"/>
+      <c r="M25" s="22"/>
+      <c r="N25" s="22"/>
+      <c r="O25" s="22"/>
+      <c r="P25" s="22"/>
+      <c r="Q25" s="24"/>
+      <c r="R25" s="22"/>
+      <c r="S25" s="22"/>
+      <c r="T25" s="24"/>
+      <c r="U25" s="22"/>
+      <c r="V25" s="22"/>
+      <c r="W25" s="22"/>
+      <c r="X25" s="22"/>
+      <c r="Y25" s="22"/>
+      <c r="Z25" s="22"/>
+      <c r="AA25" s="22"/>
+      <c r="AB25" s="24"/>
+      <c r="AC25" s="22"/>
+      <c r="AD25" s="22"/>
+      <c r="AE25" s="22"/>
+      <c r="AF25" s="22"/>
+      <c r="AG25" s="22"/>
+      <c r="AH25" s="22"/>
+      <c r="AI25" s="22"/>
+      <c r="AJ25" s="22"/>
+      <c r="AK25" s="22"/>
+      <c r="AL25" s="22"/>
+      <c r="AM25" s="22"/>
+      <c r="AN25" s="22"/>
+      <c r="AO25" s="24"/>
+      <c r="AP25" s="22"/>
+      <c r="AQ25" s="22"/>
+      <c r="AR25" s="22"/>
+      <c r="AS25" s="22"/>
+      <c r="AT25" s="22"/>
+      <c r="AU25" s="25"/>
+      <c r="AV25" s="25"/>
+      <c r="AW25" s="25"/>
+      <c r="AX25" s="22"/>
+      <c r="AY25" s="22"/>
+      <c r="AZ25" s="22"/>
+    </row>
+    <row r="26" s="23" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="22"/>
+      <c r="J26" s="22"/>
+      <c r="K26" s="22"/>
+      <c r="L26" s="24"/>
+      <c r="M26" s="22"/>
+      <c r="N26" s="22"/>
+      <c r="O26" s="22"/>
+      <c r="P26" s="22"/>
+      <c r="Q26" s="24"/>
+      <c r="R26" s="22"/>
+      <c r="S26" s="22"/>
+      <c r="T26" s="24"/>
+      <c r="U26" s="22"/>
+      <c r="V26" s="22"/>
+      <c r="W26" s="22"/>
+      <c r="X26" s="22"/>
+      <c r="Y26" s="22"/>
+      <c r="Z26" s="22"/>
+      <c r="AA26" s="22"/>
+      <c r="AB26" s="24"/>
+      <c r="AC26" s="22"/>
+      <c r="AE26" s="22"/>
+      <c r="AF26" s="22"/>
+      <c r="AG26" s="22"/>
+      <c r="AH26" s="22"/>
+      <c r="AI26" s="22"/>
+      <c r="AJ26" s="22"/>
+      <c r="AK26" s="22"/>
+      <c r="AL26" s="22"/>
+      <c r="AM26" s="22"/>
+      <c r="AN26" s="22"/>
+      <c r="AO26" s="24"/>
+      <c r="AP26" s="22"/>
+      <c r="AQ26" s="22"/>
+      <c r="AR26" s="22"/>
+      <c r="AU26" s="22"/>
+      <c r="AV26" s="22"/>
+      <c r="AW26" s="22"/>
+      <c r="AX26" s="22"/>
+      <c r="AY26" s="22"/>
+      <c r="AZ26" s="22"/>
+      <c r="BA26" s="26"/>
+      <c r="BB26" s="26"/>
+      <c r="BC26" s="22"/>
+      <c r="BD26" s="22"/>
+      <c r="BE26" s="25"/>
+    </row>
+    <row r="27" s="23" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="22"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="I27" s="22"/>
+      <c r="J27" s="22"/>
+      <c r="K27" s="22"/>
+      <c r="L27" s="24"/>
+      <c r="M27" s="22"/>
+      <c r="N27" s="22"/>
+      <c r="O27" s="22"/>
+      <c r="P27" s="22"/>
+      <c r="Q27" s="24"/>
+      <c r="R27" s="22"/>
+      <c r="S27" s="22"/>
+      <c r="T27" s="24"/>
+      <c r="U27" s="22"/>
+      <c r="V27" s="22"/>
+      <c r="W27" s="22"/>
+      <c r="X27" s="22"/>
+      <c r="Y27" s="22"/>
+      <c r="Z27" s="22"/>
+      <c r="AA27" s="22"/>
+      <c r="AB27" s="24"/>
+      <c r="AC27" s="22"/>
+      <c r="AE27" s="22"/>
+      <c r="AF27" s="22"/>
+      <c r="AG27" s="22"/>
+      <c r="AH27" s="22"/>
+      <c r="AI27" s="22"/>
+      <c r="AJ27" s="22"/>
+      <c r="AK27" s="22"/>
+      <c r="AL27" s="22"/>
+      <c r="AM27" s="22"/>
+      <c r="AN27" s="22"/>
+      <c r="AO27" s="24"/>
+      <c r="AP27" s="22"/>
+      <c r="AQ27" s="22"/>
+      <c r="AR27" s="22"/>
+      <c r="AU27" s="22"/>
+      <c r="AV27" s="22"/>
+      <c r="AW27" s="22"/>
+      <c r="AX27" s="22"/>
+      <c r="AY27" s="22"/>
+      <c r="AZ27" s="22"/>
+      <c r="BA27" s="26"/>
+      <c r="BB27" s="26"/>
+      <c r="BC27" s="22"/>
+      <c r="BD27" s="22"/>
+      <c r="BE27" s="25"/>
+    </row>
+    <row r="28" s="28" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="27"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="27"/>
+      <c r="H28" s="27"/>
+      <c r="I28" s="27"/>
+      <c r="J28" s="27"/>
+      <c r="K28" s="27"/>
+      <c r="L28" s="29"/>
+      <c r="M28" s="27"/>
+      <c r="N28" s="27"/>
+      <c r="O28" s="27"/>
+      <c r="P28" s="27"/>
+      <c r="Q28" s="29"/>
+      <c r="R28" s="27"/>
+      <c r="S28" s="27"/>
+      <c r="T28" s="29"/>
+      <c r="U28" s="27"/>
+      <c r="V28" s="27"/>
+      <c r="W28" s="27"/>
+      <c r="X28" s="27"/>
+      <c r="Y28" s="27"/>
+      <c r="Z28" s="27"/>
+      <c r="AA28" s="27"/>
+      <c r="AB28" s="29"/>
+      <c r="AC28" s="27"/>
+      <c r="AD28" s="27"/>
+      <c r="AE28" s="27"/>
+      <c r="AF28" s="27"/>
+      <c r="AG28" s="27"/>
+      <c r="AH28" s="27"/>
+      <c r="AI28" s="27"/>
+      <c r="AJ28" s="27"/>
+      <c r="AK28" s="27"/>
+      <c r="AL28" s="27"/>
+      <c r="AM28" s="27"/>
+      <c r="AN28" s="27"/>
+      <c r="AO28" s="29"/>
+      <c r="AP28" s="27"/>
+      <c r="AQ28" s="27"/>
+      <c r="AR28" s="27"/>
+      <c r="AS28" s="27"/>
+      <c r="AT28" s="27"/>
+      <c r="AU28" s="19"/>
+      <c r="AV28" s="19"/>
+      <c r="AW28" s="19"/>
+      <c r="AX28" s="30"/>
+      <c r="AY28" s="30"/>
+      <c r="AZ28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="AU29" s="22"/>
-      <c r="AV29" s="22"/>
-      <c r="AW29" s="22"/>
-      <c r="AX29" s="22"/>
-      <c r="AY29" s="22"/>
-      <c r="AZ29" s="22"/>
+      <c r="AU29" s="20"/>
+      <c r="AV29" s="20"/>
+      <c r="AW29" s="20"/>
+      <c r="AX29" s="20"/>
+      <c r="AY29" s="20"/>
+      <c r="AZ29" s="20"/>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2355,7 +2221,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.60546875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2373,7 +2239,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.60546875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>